<commit_message>
Estilo de tablas: quitar líneas de cuerpo, dejar solo header/paneles/cierre
- tabla_aer(): cuerpo en blanco (sin borde por fila); línea superior fina solo en
  cada panel (autodetectados por 'Panel ' en col 1), header y cierre.
- numFmt '@' en celdas de datos: suprime el aviso verde de Excel (texto a propósito).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/tab1_descriptiva.xlsx
+++ b/outputs/tables/tab1_descriptiva.xlsx
@@ -294,7 +294,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="@"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <sz val="11"/>
@@ -358,19 +360,19 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="FF888888"/>
       </bottom>
     </border>
     <border>
-      <bottom style="thin">
+      <top style="thin">
         <color rgb="FF888888"/>
-      </bottom>
+      </top>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -382,13 +384,19 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -838,25 +846,25 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" s="5" t="s">
+      <c r="C8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>8</v>
       </c>
     </row>
@@ -930,25 +938,25 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H12" s="5" t="s">
+      <c r="C12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1068,7 +1076,7 @@
       </c>
     </row>
     <row r="18" ht="102" customHeight="1">
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="10" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tabla 1: reportar mediana [IQR] en vez de media (DE) por la fuerte asimetría
Los subsidios son muy asimétricos (~1/3 de país-año en cero, pocos países concentran
montos altos): la media engañaba (DE > media, media = 20x la mediana). Se reporta mediana
con rango intercuartílico [P25, P75]. Nota al pie aclara unidad (USD miles de millones) y
el motivo. Unidades verificadas contra la fuente: subsidio/PIB = expl_pctgdp (cuadra).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/tab1_descriptiva.xlsx
+++ b/outputs/tables/tab1_descriptiva.xlsx
@@ -65,121 +65,121 @@
     <t xml:space="preserve">  Explícito</t>
   </si>
   <si>
-    <t xml:space="preserve">1.45 (3.79)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.91 (6.03)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.55 (2.20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.35 (3.62)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.33 (5.53)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.21 (2.67)</t>
+    <t xml:space="preserve">0.07 [0.00, 0.52]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.23 [0.60, 6.22]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.02 [0.00, 0.19]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.07 [0.00, 0.51]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.15 [0.01, 0.62]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.14 [0.01, 0.52]</t>
   </si>
   <si>
     <t xml:space="preserve">  Implícito</t>
   </si>
   <si>
-    <t xml:space="preserve">7.34 (14.46)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14.93 (20.68)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.89 (10.74)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.97 (13.49)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.41 (19.43)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.72 (15.23)</t>
+    <t xml:space="preserve">1.29 [0.17, 6.59]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.41 [1.50, 17.71]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.74 [0.04, 2.19]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.19 [0.17, 6.94]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.69 [0.24, 6.58]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.34 [0.30, 6.12]</t>
   </si>
   <si>
     <t xml:space="preserve">  Total</t>
   </si>
   <si>
-    <t xml:space="preserve">9.53 (18.38)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20.48 (26.30)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.00 (13.23)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.05 (17.07)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.60 (25.74)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.67 (18.43)</t>
+    <t xml:space="preserve">1.45 [0.23, 10.31]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.67 [2.23, 24.96]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.85 [0.05, 2.44]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.29 [0.22, 10.24]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.89 [0.31, 12.18]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.65 [0.35, 10.18]</t>
   </si>
   <si>
     <t xml:space="preserve">Panel B. Subsidios (% del PIB)</t>
   </si>
   <si>
-    <t xml:space="preserve">1.15 (2.45)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.59 (4.23)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.51 (0.99)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.03 (2.23)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.84 (3.56)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.29 (2.57)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.20 (2.37)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.89 (2.71)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.33 (1.40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.03 (2.34)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.03 (2.44)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.46 (2.34)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.44 (4.66)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.54 (6.70)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.80 (1.80)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.17 (4.47)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.90 (5.71)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.77 (4.62)</t>
+    <t xml:space="preserve">0.30 [0.06, 1.04]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.17 [0.91, 4.16]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.14 [0.03, 0.46]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.24 [0.06, 0.95]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.43 [0.07, 1.96]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.34 [0.09, 1.15]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.72 [1.66, 4.17]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.24 [4.37, 6.60]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.13 [1.32, 3.30]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.63 [1.53, 4.01]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.38 [2.19, 5.33]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.80 [1.65, 4.77]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.22 [1.90, 5.10]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.50 [4.95, 10.12]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.62 [1.51, 3.80]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.03 [1.76, 4.64]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.69 [2.54, 7.57]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.29 [1.97, 5.17]</t>
   </si>
   <si>
     <t xml:space="preserve">Panel C. Canal de precios y contexto fiscal</t>
@@ -188,85 +188,85 @@
     <t xml:space="preserve">  Brecha de precio gasolina</t>
   </si>
   <si>
-    <t xml:space="preserve">0.29 (0.41)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.19 (0.36)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.41 (0.32)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.31 (0.41)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.16 (0.42)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.26 (0.39)</t>
+    <t xml:space="preserve">0.28 [0.05, 0.53]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.16 [-0.43, 0.06]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.38 [0.18, 0.58]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.32 [0.12, 0.54]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.18 [0.01, 0.36]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.24 [0.06, 0.47]</t>
   </si>
   <si>
     <t xml:space="preserve">  Brecha de precio diésel</t>
   </si>
   <si>
-    <t xml:space="preserve">0.24 (0.32)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.10 (0.38)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.33 (0.24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.25 (0.31)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.11 (0.37)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.31 (0.36)</t>
+    <t xml:space="preserve">0.27 [0.06, 0.44]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.14 [-0.44, 0.21]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.31 [0.14, 0.49]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.28 [0.08, 0.43]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.12 [0.00, 0.31]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.38 [0.12, 0.55]</t>
   </si>
   <si>
     <t xml:space="preserve">  Balance fiscal (% PIB) (a)</t>
   </si>
   <si>
-    <t xml:space="preserve">-3.14 (2.91)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.01 (2.57)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.92 (2.96)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3.27 (3.00)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.43 (2.36)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.56 (2.41)</t>
+    <t xml:space="preserve">-2.79 [-4.46, -1.27]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.35 [-5.50, -2.16]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.62 [-4.40, -1.03]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.78 [-4.93, -1.31]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.73 [-4.43, -0.05]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.10 [-3.65, -1.85]</t>
   </si>
   <si>
     <t xml:space="preserve">  Ingreso público (% PIB) (a)</t>
   </si>
   <si>
-    <t xml:space="preserve">21.77 (5.66)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.05 (4.98)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21.02 (5.55)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21.63 (5.68)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22.87 (5.81)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22.11 (5.53)</t>
+    <t xml:space="preserve">21.51 [17.56, 26.07]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.26 [19.36, 29.15]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.75 [17.00, 25.42]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.50 [17.47, 25.63]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.46 [18.11, 27.88]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.51 [17.78, 26.05]</t>
   </si>
   <si>
     <t xml:space="preserve">N (país-año)</t>
@@ -287,7 +287,7 @@
     <t xml:space="preserve">34</t>
   </si>
   <si>
-    <t xml:space="preserve">Notas. Estadística descriptiva del panel país-año de América Latina y el Caribe, 2015-2023. Cada celda reporta la media entre países con la desviación estándar entre paréntesis. Las columnas desagregan la muestra completa (1) por condición de exportador neto de hidrocarburos (2)-(3) y por período relativo al choque petrolero de 2022 (4)-(6); exportadores netos: Bolivia, Colombia, Ecuador, Guyana, México, Trinidad y Tobago y Venezuela. (a) Cobertura parcial: la fuente no reporta el dato para todos los país-año. Las brechas de precio son el precio al consumidor menos el costo de suministro. Fuentes: IMF Fossil Fuel Subsidies Database y World Bank (WDI).</t>
+    <t xml:space="preserve">Notas. Estadística descriptiva del panel país-año de América Latina y el Caribe, 2015-2023. Cada celda reporta la mediana entre países con el rango intercuartílico [P25, P75] entre corchetes; los subsidios en niveles están en USD miles de millones. Se usa la mediana por la fuerte asimetría de la distribución (cerca de un tercio de los país-año no aplican subsidio explícito). Las columnas desagregan la muestra completa (1) por condición de exportador neto de hidrocarburos (2)-(3) y por período relativo al choque petrolero de 2022 (4)-(6); exportadores netos: Bolivia, Colombia, Ecuador, Guyana, México, Trinidad y Tobago y Venezuela. (a) Cobertura parcial: la fuente no reporta el dato para todos los país-año. Las brechas de precio son el precio al consumidor menos el costo de suministro. Fuentes: IMF Fossil Fuel Subsidies Database y World Bank (WDI).</t>
   </si>
 </sst>
 </file>
@@ -1075,7 +1075,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" ht="102" customHeight="1">
+    <row r="18" ht="130" customHeight="1">
       <c r="B18" s="10" t="s">
         <v>91</v>
       </c>

</xml_diff>

<commit_message>
Descriptivas: tablas con paneles encajonados + fila N, y figura de la ruptura 2022
Tablas (T1 anual, T2 por país):
- Fila N por panel, encajonada (línea arriba thin + cierre medium), sin fila de aire
- Paneles con apertura/cierre medium; header sin triángulos verdes (numFmt texto)
- Nombres de país traducidos al español (catálogo PAIS_ES en config.R)
- Notas: criterio de exportador neto (exposición fiscal, no producción) + lista de países
- T2 desagregada por año (2015-2023) + cambio del choque

Figura fig1_ruptura.png (grid 2x2, color WB, PNG 300 dpi):
- Línea vertical en 2022 (convención event-study para evento puntual)
- Valores anotados en años clave; nota al pie compuesta dentro del PNG
- Helper save_fig_png() en config.R

01_variables.py: documenta el criterio de exportador neto (exposición fiscal neta).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/tab1_descriptiva.xlsx
+++ b/outputs/tables/tab1_descriptiva.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
   <si>
     <t xml:space="preserve">Tabla 1. Evolución anual de los subsidios a combustibles fósiles (2015-2023)</t>
   </si>
@@ -170,6 +170,12 @@
     <t xml:space="preserve">4.77</t>
   </si>
   <si>
+    <t xml:space="preserve">  N (países)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34</t>
+  </si>
+  <si>
     <t xml:space="preserve">Panel B. Exportadores netos de hidrocarburos</t>
   </si>
   <si>
@@ -278,6 +284,9 @@
     <t xml:space="preserve">6.44</t>
   </si>
   <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
     <t xml:space="preserve">Panel C. Importadores netos</t>
   </si>
   <si>
@@ -386,15 +395,22 @@
     <t xml:space="preserve">3.83</t>
   </si>
   <si>
-    <t xml:space="preserve">Notas. Subsidios a combustibles fósiles en América Latina y el Caribe (34 países), por año y grupo de exposición, alrededor del choque petrolero de 2022. Cada celda es la suma del grupo en el año: en USD miles de millones (USD bn) y como porcentaje del PIB agregado del grupo. Exportadores netos: Bolivia, Colombia, Ecuador, Guyana, México, Trinidad y Tobago y Venezuela; el resto son importadores netos. Fuente: IMF Fossil Fuel Subsidies Database.</t>
+    <t xml:space="preserve">27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notas. Subsidios a combustibles fósiles en América Latina y el Caribe, por año y grupo de exposición, alrededor del choque petrolero de 2022. Cada celda es la suma del grupo en el año: en USD miles de millones (USD bn) y como porcentaje del PIB agregado del grupo. El subsidio explícito mide la brecha entre el precio al consumidor y el costo de suministro; el total suma además el componente implícito (externalidades no internalizadas e IVA no aplicado). El explícito es el que reacciona al choque. La clasificación es por exposición fiscal neta al precio del petróleo, no por producción: en los exportadores netos el alza del Brent infla la renta petrolera que financia el subsidio, mientras que en los importadores netos encarece el costo de suministro y agrava el gasto en subsidios. Argentina (importador neto de energía en el período) y Brasil (importa los derivados refinados que se subsidian) se clasifican como importadores. Panel A, Total LATAM (N = 34 países). Panel B, exportadores netos de hidrocarburos (N = 7): Bolivia, Colombia, Ecuador, Guyana, México, Trinidad y Tobago y Venezuela. Panel C, importadores netos (N = 27): Antigua y Barbuda, Argentina, Aruba, Bahamas, Barbados, Belice, Brasil, Chile, Costa Rica, Dominica, El Salvador, Granada, Guatemala, Haití, Honduras, Jamaica, Nicaragua, Panamá, Paraguay, Perú, Puerto Rico, República Dominicana, San Cristóbal y Nieves, San Vicente y las Granadinas, Santa Lucía, Surinam, Uruguay. Fuente: IMF Fossil Fuel Subsidies Database.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="5">
     <numFmt numFmtId="166" formatCode="@"/>
+    <numFmt numFmtId="167" formatCode="@"/>
+    <numFmt numFmtId="170" formatCode="0"/>
+    <numFmt numFmtId="168" formatCode="0"/>
+    <numFmt numFmtId="169" formatCode="0"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -458,12 +474,15 @@
       </bottom>
     </border>
     <border>
-      <bottom style="thin">
+      <top style="thin">
+        <color rgb="FF888888"/>
+      </top>
+      <bottom style="medium">
         <color rgb="FF888888"/>
       </bottom>
     </border>
     <border>
-      <top style="thin">
+      <top style="medium">
         <color rgb="FF888888"/>
       </top>
     </border>
@@ -471,28 +490,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -839,34 +864,34 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="K3" s="4" t="s">
+      <c r="C3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="K3" s="8" t="s">
         <v>12</v>
       </c>
     </row>
@@ -999,333 +1024,429 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>12</v>
+      <c r="C8" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="B9" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>61</v>
+      <c r="C9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="J10" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="K10" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J11" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E11" s="4" t="s">
+      <c r="K11" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E12" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="H13" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="I13" s="4" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="7" t="s">
+      <c r="J13" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>12</v>
+      <c r="K13" s="4" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="E14" s="4" t="s">
+      <c r="B14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K14" s="10" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>106</v>
+      <c r="C15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="F16" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="G16" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="H16" s="4" t="s">
+      <c r="D18" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="E18" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="G18" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H18" s="4" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="5" t="s">
+      <c r="I18" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="F17" s="6" t="s">
+      <c r="C19" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="D19" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="E19" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="F19" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="G19" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="H19" s="4" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="B18" s="9" t="s">
+      <c r="I19" s="4" t="s">
         <v>124</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" ht="158" customHeight="1">
+      <c r="B21" s="11" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B18:K18"/>
+    <mergeCell ref="B21:K21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Consolidar subsidios en Tabla 1: añadir implícito, eliminar Tabla 3
La Tabla 3 repetía explícito/total que ya estaban en la Tabla 1. Se absorbe
su único aporte único (el subsidio implícito) como filas nuevas en cada panel
de la Tabla 1 — explícito/implícito/total en USD bn y % PIB, año por año.
Así toda la dinámica de subsidios vive en un solo lugar, completa y temporal,
y se ve que el implícito domina en nivel pero apenas reacciona al choque
(a diferencia del explícito). El Brent ya figura como tratamiento en la Fig 1.

Renumera figuras a 03-04 para numeración consecutiva tras quitar la Tabla 3.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/tab1_descriptiva.xlsx
+++ b/outputs/tables/tab1_descriptiva.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="180">
   <si>
     <t xml:space="preserve">Tabla 1. Evolución anual de los subsidios a combustibles fósiles (2015-2023)</t>
   </si>
@@ -83,6 +83,36 @@
     <t xml:space="preserve">41.3</t>
   </si>
   <si>
+    <t xml:space="preserve">  Implícito (USD bn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">192.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">197.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">197.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">204.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">204.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">158.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">224.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">282.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">231.6</t>
+  </si>
+  <si>
     <t xml:space="preserve">  Total (USD bn)</t>
   </si>
   <si>
@@ -140,6 +170,36 @@
     <t xml:space="preserve">0.68</t>
   </si>
   <si>
+    <t xml:space="preserve">  Implícito (% PIB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.91</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.87</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.97</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.81</t>
+  </si>
+  <si>
     <t xml:space="preserve">  Total (% PIB)</t>
   </si>
   <si>
@@ -155,9 +215,6 @@
     <t xml:space="preserve">4.12</t>
   </si>
   <si>
-    <t xml:space="preserve">3.92</t>
-  </si>
-  <si>
     <t xml:space="preserve">3.63</t>
   </si>
   <si>
@@ -206,6 +263,30 @@
     <t xml:space="preserve">24.0</t>
   </si>
   <si>
+    <t xml:space="preserve">110.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">117.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">110.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">106.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">97.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">71.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">89.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">131.2</t>
+  </si>
+  <si>
     <t xml:space="preserve">149.0</t>
   </si>
   <si>
@@ -257,6 +338,33 @@
     <t xml:space="preserve">1.10</t>
   </si>
   <si>
+    <t xml:space="preserve">4.81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.88</t>
+  </si>
+  <si>
     <t xml:space="preserve">6.46</t>
   </si>
   <si>
@@ -272,9 +380,6 @@
     <t xml:space="preserve">5.65</t>
   </si>
   <si>
-    <t xml:space="preserve">4.88</t>
-  </si>
-  <si>
     <t xml:space="preserve">6.28</t>
   </si>
   <si>
@@ -317,6 +422,33 @@
     <t xml:space="preserve">17.3</t>
   </si>
   <si>
+    <t xml:space="preserve">81.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">87.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">106.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">87.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">135.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">151.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">125.3</t>
+  </si>
+  <si>
     <t xml:space="preserve">116.3</t>
   </si>
   <si>
@@ -368,12 +500,33 @@
     <t xml:space="preserve">0.44</t>
   </si>
   <si>
+    <t xml:space="preserve">1.90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.94</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.21</t>
+  </si>
+  <si>
     <t xml:space="preserve">2.71</t>
   </si>
   <si>
-    <t xml:space="preserve">2.55</t>
-  </si>
-  <si>
     <t xml:space="preserve">2.31</t>
   </si>
   <si>
@@ -398,7 +551,7 @@
     <t xml:space="preserve">27</t>
   </si>
   <si>
-    <t xml:space="preserve">Notas. Subsidios a combustibles fósiles en América Latina y el Caribe, por año y grupo de exposición, alrededor del choque petrolero de 2022. Cada celda es la suma del grupo en el año: en USD miles de millones (USD bn) y como porcentaje del PIB agregado del grupo. El subsidio explícito mide la brecha entre el precio al consumidor y el costo de suministro; el total suma además el componente implícito (externalidades no internalizadas e IVA no aplicado). El explícito es el que reacciona al choque. La clasificación es por exposición fiscal neta al precio del petróleo, no por producción: en los exportadores netos el alza del Brent infla la renta petrolera que financia el subsidio, mientras que en los importadores netos encarece el costo de suministro y agrava el gasto en subsidios. Argentina (importador neto de energía en el período) y Brasil (importa los derivados refinados que se subsidian) se clasifican como importadores. Panel A, Total LATAM (N = 34 países). Panel B, exportadores netos de hidrocarburos (N = 7): Bolivia, Colombia, Ecuador, Guyana, México, Trinidad y Tobago y Venezuela. Panel C, importadores netos (N = 27): Antigua y Barbuda, Argentina, Aruba, Bahamas, Barbados, Belice, Brasil, Chile, Costa Rica, Dominica, El Salvador, Granada, Guatemala, Haití, Honduras, Jamaica, Nicaragua, Panamá, Paraguay, Perú, Puerto Rico, República Dominicana, San Cristóbal y Nieves, San Vicente y las Granadinas, Santa Lucía, Surinam, Uruguay. Fuente: IMF Fossil Fuel Subsidies Database.</t>
+    <t xml:space="preserve">Notas. Subsidios a combustibles fósiles en América Latina y el Caribe, por año y grupo de exposición, alrededor del choque petrolero de 2022. Cada celda es la suma del grupo en el año: en USD miles de millones (USD bn) y como porcentaje del PIB agregado del grupo. El subsidio explícito mide la brecha entre el precio al consumidor y el costo de suministro; el implícito recoge las externalidades no internalizadas y el IVA no aplicado; el total es la suma de ambos. El explícito es el componente que reacciona al choque en el corto plazo; el implícito depende del volumen consumido y de parámetros de daño ambiental, no del precio internacional. El implícito (y, por tanto, el total) no está estimado para todos los país-año. La clasificación es por exposición fiscal neta al precio del petróleo, no por producción: en los exportadores netos el alza del Brent infla la renta petrolera que financia el subsidio, mientras que en los importadores netos encarece el costo de suministro y agrava el gasto en subsidios. Argentina (importador neto de energía en el período) y Brasil (importa los derivados refinados que se subsidian) se clasifican como importadores. Panel A, Total LATAM (N = 34 países). Panel B, exportadores netos de hidrocarburos (N = 7): Bolivia, Colombia, Ecuador, Guyana, México, Trinidad y Tobago y Venezuela. Panel C, importadores netos (N = 27): Antigua y Barbuda, Argentina, Aruba, Bahamas, Barbados, Belice, Brasil, Chile, Costa Rica, Dominica, El Salvador, Granada, Guatemala, Haití, Honduras, Jamaica, Nicaragua, Panamá, Paraguay, Perú, Puerto Rico, República Dominicana, San Cristóbal y Nieves, San Vicente y las Granadinas, Santa Lucía, Surinam, Uruguay. Fuente: IMF Fossil Fuel Subsidies Database.</t>
   </si>
 </sst>
 </file>
@@ -982,39 +1135,39 @@
         <v>39</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="J7" s="4" t="s">
         <v>50</v>
@@ -1024,429 +1177,621 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D10" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E10" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F10" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G10" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="H10" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="I8" s="9" t="n">
+      <c r="I10" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="J8" s="9" t="n">
+      <c r="J10" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="K8" s="9" t="n">
+      <c r="K10" s="9" t="n">
         <v>34</v>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
     <row r="11">
-      <c r="B11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>72</v>
+      <c r="B11" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H13" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="K13" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="I13" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C14" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="E14" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="F14" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="G14" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="I14" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="J14" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K14" s="10" t="n">
-        <v>7</v>
+      <c r="B14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="K15" s="8" t="s">
-        <v>12</v>
+      <c r="B15" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K18" s="10" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="K17" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="3" t="s">
+      <c r="C21" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="J19" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="K19" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="5" t="s">
+      <c r="C22" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C24" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D26" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="E20" s="6" t="n">
+      <c r="E26" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F26" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G26" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="H20" s="6" t="n">
+      <c r="H26" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="I20" s="6" t="n">
+      <c r="I26" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="J20" s="6" t="n">
+      <c r="J26" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="K20" s="6" t="n">
+      <c r="K26" s="6" t="n">
         <v>27</v>
       </c>
     </row>
-    <row r="21" ht="158" customHeight="1">
-      <c r="B21" s="11" t="s">
-        <v>128</v>
+    <row r="27" ht="172" customHeight="1">
+      <c r="B27" s="11" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B21:K21"/>
+    <mergeCell ref="B27:K27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>